<commit_message>
feat: Pivot-Tabelle zum Dashboard_Template hinzugefügt
</commit_message>
<xml_diff>
--- a/Systemdaten/Dashboard_Template.xlsx
+++ b/Systemdaten/Dashboard_Template.xlsx
@@ -1,35 +1,95 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dangi\Desktop\Buchhaltung\Systemdaten\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3B20180-2C80-4946-902C-8EF89B94D848}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rohdaten" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
+    <sheet name="Rohdaten" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
+  <pivotCaches>
+    <pivotCache cacheId="4" r:id="rId3"/>
+  </pivotCaches>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+  <si>
+    <t>Sektorenanalyse Dashboard</t>
+  </si>
+  <si>
+    <t>Hier kannst du später Pivot-Tabellen und Diagramme einfügen, die auf den 'Rohdaten' basieren.</t>
+  </si>
+  <si>
+    <t>Datei</t>
+  </si>
+  <si>
+    <t>Datum</t>
+  </si>
+  <si>
+    <t>Nummer</t>
+  </si>
+  <si>
+    <t>Lieferant</t>
+  </si>
+  <si>
+    <t>Beschreibung</t>
+  </si>
+  <si>
+    <t>Menge</t>
+  </si>
+  <si>
+    <t>Gesamtpreis</t>
+  </si>
+  <si>
+    <t>Fleischart</t>
+  </si>
+  <si>
+    <t>Rind</t>
+  </si>
+  <si>
+    <t>Schwein</t>
+  </si>
+  <si>
+    <t>Zeilenbeschriftungen</t>
+  </si>
+  <si>
+    <t>(Leer)</t>
+  </si>
+  <si>
+    <t>Gesamtergebnis</t>
+  </si>
+  <si>
+    <t>Summe von Gesamtpreis</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -47,82 +107,161 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Tobias Weiss" refreshedDate="46225.027588425924" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{71E04CBA-7401-4C6B-815B-7A8D2AB0B51C}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A1:H9998" sheet="Rohdaten"/>
+  </cacheSource>
+  <cacheFields count="8">
+    <cacheField name="Datei" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Datum" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Nummer" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="123" maxValue="124"/>
+    </cacheField>
+    <cacheField name="Lieferant" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Beschreibung" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Menge" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="5" maxValue="10"/>
+    </cacheField>
+    <cacheField name="Gesamtpreis" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="45" maxValue="150.5"/>
+    </cacheField>
+    <cacheField name="Fleischart" numFmtId="0">
+      <sharedItems containsBlank="1" count="3">
+        <s v="Rind"/>
+        <s v="Schwein"/>
+        <m/>
+      </sharedItems>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="3">
+  <r>
+    <s v="test.xml"/>
+    <s v="01.01.2026"/>
+    <n v="123"/>
+    <s v="Metzger Max"/>
+    <s v="Rinderhack"/>
+    <n v="10"/>
+    <n v="150.5"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <s v="test2.xml"/>
+    <s v="02.01.2026"/>
+    <n v="124"/>
+    <s v="Metzger Max"/>
+    <s v="Schweinehals"/>
+    <n v="5"/>
+    <n v="45"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <x v="2"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{38372466-F377-4E89-B50F-C39A77110D4B}" name="AusgabenNachFleischart" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A5:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="8">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Summe von Gesamtpreis" fld="6" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -409,26 +548,60 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Sektorenanalyse Dashboard</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Hier kannst du später Pivot-Tabellen und Diagramme einfügen, die auf den 'Rohdaten' basieren.</t>
-        </is>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="3">
+        <v>150.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="3"/>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="3">
+        <v>195.5</v>
       </c>
     </row>
   </sheetData>
@@ -437,19 +610,34 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Rechnung</t>
-        </is>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>